<commit_message>
Proofread loan clean-up plan: clarify notes, add 43% coverage item, consistent GL row refs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y5ymXYu4DLEyfkehRGcSfY
</commit_message>
<xml_diff>
--- a/output/GAEA_Loan_Cleanup_Plan.xlsx
+++ b/output/GAEA_Loan_Cleanup_Plan.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="450">
   <si>
     <t xml:space="preserve">800 Super GAEA - Loan &amp; Interest Clean-up (responsAbility + Healthier loans)</t>
   </si>
@@ -279,6 +279,9 @@
     <t xml:space="preserve">Interest paid by 800S for FHL (13-Jun-2024)</t>
   </si>
   <si>
+    <t xml:space="preserve">Same (bank slip 107,674.43 less USD 1,163.29 moved to principal).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Principal paid by 800S, each loan (28-Jun-2024)</t>
   </si>
   <si>
@@ -312,7 +315,7 @@
     <t xml:space="preserve">rA default interest</t>
   </si>
   <si>
-    <t xml:space="preserve">rA unpaid interest</t>
+    <t xml:space="preserve">rA unpaid interest (client figure worked out from its daily schedule)</t>
   </si>
   <si>
     <t xml:space="preserve">Different</t>
@@ -333,13 +336,13 @@
     <t xml:space="preserve">2023 interest - rA</t>
   </si>
   <si>
-    <t xml:space="preserve">Small: we split the Sep-23 to Mar-24 period by days/182; the lender uses days/365 and /366 for 2024.</t>
+    <t xml:space="preserve">Small: different way of splitting the Sep-23 to Mar-24 interest between 2023 and 2024 (we used days/182 of the notice amount; the lender uses days/365, days/366 for 2024, and its month-end cut-off).</t>
   </si>
   <si>
     <t xml:space="preserve">2023 interest - FHL</t>
   </si>
   <si>
-    <t xml:space="preserve">Small: same day-count reason.</t>
+    <t xml:space="preserve">Small: same splitting reason as above.</t>
   </si>
   <si>
     <t xml:space="preserve">2024 interest - rA</t>
@@ -438,7 +441,7 @@
     <t xml:space="preserve">Catch-up accrual still needed in JV books to 30-Sep-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Per client file: interest 177,238.03 + penalty 33,588.50.</t>
+    <t xml:space="preserve">Per client file: interest 177,238.03 + penalty 33,588.50 (adds to .53 because of rounding; client total is 210,826.52).</t>
   </si>
   <si>
     <t xml:space="preserve">Penalty waiver remark ("RA agreed to waive penalties")</t>
@@ -453,6 +456,18 @@
     <t xml:space="preserve">Lender's 2026 figure still includes default interest. Waiver must be documented.</t>
   </si>
   <si>
+    <t xml:space="preserve">Share of interest actually covered by 800S in June 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About 43% (rA 42.9% / FHL 43.3%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51% assumed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under the lender method the June 2024 payment covered ~43% of interest + default owed at 13-Jun-2024, not 51%. Amount paid is the same; only the % differs.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Amendment Agreement (drafts Jul-2026)</t>
   </si>
   <si>
@@ -516,7 +531,7 @@
     <t xml:space="preserve">Entries in QuickBooks to DELETE or EDIT</t>
   </si>
   <si>
-    <t xml:space="preserve">DELETE = remove the whole transaction. EDIT = open the transaction and change only the account named (do NOT delete - these are real bank/tax payments). GL row = row number in the GL file you sent.</t>
+    <t xml:space="preserve">DELETE = remove the whole transaction. EDIT = open the transaction and change only the account named (do NOT delete - these are real bank/tax payments). GL row = row number in the GL file you sent (for journal entries: the first line of the entry in that account).</t>
   </si>
   <si>
     <t xml:space="preserve">Action</t>
@@ -837,7 +852,7 @@
     <t xml:space="preserve">Total 14% WHT already paid, moved 20010 -&gt; 63025</t>
   </si>
   <si>
-    <t xml:space="preserve">(the 2 partial-edit entries count only their 4,082.26 WHT line)</t>
+    <t xml:space="preserve">(13 WHT entries + the 4,082.26 WHT line in each of ADJ2305-002 and ADJ2306-001)</t>
   </si>
   <si>
     <t xml:space="preserve">Correcting entries to post (after the deletions and edits in tab 2)</t>
@@ -861,7 +876,7 @@
     <t xml:space="preserve">Long-term liability</t>
   </si>
   <si>
-    <t xml:space="preserve">Accounts 20259, 20260, 20261, 20262 already exist - keep using them.</t>
+    <t xml:space="preserve">Accounts 20259, 20260, 20261, 20262 already exist - keep using them. (20261 is spelt "responsibility" in QuickBooks - same account; you may correct the spelling.)</t>
   </si>
   <si>
     <t xml:space="preserve">Loan payable - Healthier</t>
@@ -2298,7 +2313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2709,7 +2724,7 @@
         <v>55</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,7 +2732,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C22" s="15" t="n">
         <v>765000</v>
@@ -2733,7 +2748,7 @@
         <v>55</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2741,7 +2756,7 @@
         <v>17</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C23" s="15" t="n">
         <v>735000</v>
@@ -2757,7 +2772,7 @@
         <v>55</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2765,7 +2780,7 @@
         <v>18</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C24" s="15" t="n">
         <v>1745676.83</v>
@@ -2781,13 +2796,13 @@
         <v>55</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11"/>
       <c r="B25" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
@@ -2800,7 +2815,7 @@
         <v>19</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C26" s="15" t="n">
         <v>192181.77</v>
@@ -2816,7 +2831,7 @@
         <v>55</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2824,7 +2839,7 @@
         <v>20</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C27" s="15" t="n">
         <v>16663.6</v>
@@ -2848,7 +2863,7 @@
         <v>21</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C28" s="15" t="n">
         <v>16992.36</v>
@@ -2872,7 +2887,7 @@
         <v>22</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C29" s="19" t="n">
         <v>195086.71</v>
@@ -2885,16 +2900,16 @@
         <v>-1971.30000000002</v>
       </c>
       <c r="F29" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11"/>
       <c r="B30" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C30" s="11"/>
       <c r="D30" s="11"/>
@@ -2907,7 +2922,7 @@
         <v>23</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C31" s="15" t="n">
         <v>47227.81</v>
@@ -2931,7 +2946,7 @@
         <v>24</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C32" s="15" t="n">
         <v>47227.81</v>
@@ -2950,12 +2965,12 @@
         <v>69</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="n">
         <v>25</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C33" s="19" t="n">
         <v>184772.83</v>
@@ -2968,10 +2983,10 @@
         <v>70.0399999999791</v>
       </c>
       <c r="F33" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2979,7 +2994,7 @@
         <v>26</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C34" s="19" t="n">
         <v>184002.11</v>
@@ -2992,10 +3007,10 @@
         <v>70.9499999999825</v>
       </c>
       <c r="F34" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G34" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3003,7 +3018,7 @@
         <v>27</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C35" s="19" t="n">
         <v>154706.19</v>
@@ -3016,10 +3031,10 @@
         <v>-17258.96</v>
       </c>
       <c r="F35" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G35" s="18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3027,7 +3042,7 @@
         <v>28</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C36" s="19" t="n">
         <v>154818.66</v>
@@ -3040,10 +3055,10 @@
         <v>-1519.03</v>
       </c>
       <c r="F36" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G36" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3051,7 +3066,7 @@
         <v>29</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C37" s="19" t="n">
         <v>95192.37</v>
@@ -3064,10 +3079,10 @@
         <v>-21743.44</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G37" s="18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3075,7 +3090,7 @@
         <v>30</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C38" s="19" t="n">
         <v>95034.22</v>
@@ -3088,10 +3103,10 @@
         <v>-7871.23</v>
       </c>
       <c r="F38" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G38" s="18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3099,7 +3114,7 @@
         <v>31</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C39" s="19" t="n">
         <v>201893.06</v>
@@ -3112,10 +3127,10 @@
         <v>-17188.92</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G39" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3123,7 +3138,7 @@
         <v>32</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C40" s="19" t="n">
         <v>201381.69</v>
@@ -3136,16 +3151,16 @@
         <v>-1448.07999999999</v>
       </c>
       <c r="F40" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G40" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11"/>
       <c r="B41" s="12" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C41" s="11"/>
       <c r="D41" s="11"/>
@@ -3158,20 +3173,20 @@
         <v>33</v>
       </c>
       <c r="B42" s="22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E42" s="22"/>
       <c r="F42" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3179,20 +3194,20 @@
         <v>34</v>
       </c>
       <c r="B43" s="22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D43" s="22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E43" s="22"/>
       <c r="F43" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G43" s="22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3200,20 +3215,20 @@
         <v>35</v>
       </c>
       <c r="B44" s="22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D44" s="22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E44" s="22"/>
       <c r="F44" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3221,7 +3236,7 @@
         <v>36</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C45" s="24" t="n">
         <v>182876.04</v>
@@ -3229,10 +3244,10 @@
       <c r="D45" s="22"/>
       <c r="E45" s="22"/>
       <c r="F45" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3240,7 +3255,7 @@
         <v>37</v>
       </c>
       <c r="B46" s="22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C46" s="24" t="n">
         <v>684589.1</v>
@@ -3248,10 +3263,10 @@
       <c r="D46" s="22"/>
       <c r="E46" s="22"/>
       <c r="F46" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3259,7 +3274,7 @@
         <v>38</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C47" s="24" t="n">
         <v>2202977.49</v>
@@ -3267,10 +3282,10 @@
       <c r="D47" s="22"/>
       <c r="E47" s="22"/>
       <c r="F47" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G47" s="22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3278,7 +3293,7 @@
         <v>39</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C48" s="24" t="n">
         <v>519656.72</v>
@@ -3286,10 +3301,10 @@
       <c r="D48" s="22"/>
       <c r="E48" s="22"/>
       <c r="F48" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3297,7 +3312,7 @@
         <v>40</v>
       </c>
       <c r="B49" s="22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C49" s="24" t="n">
         <v>210826.52</v>
@@ -3305,10 +3320,10 @@
       <c r="D49" s="22"/>
       <c r="E49" s="22"/>
       <c r="F49" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G49" s="22" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3316,20 +3331,20 @@
         <v>41</v>
       </c>
       <c r="B50" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E50" s="22"/>
       <c r="F50" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3337,74 +3352,74 @@
         <v>42</v>
       </c>
       <c r="B51" s="22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D51" s="22" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="E51" s="22"/>
       <c r="F51" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="21" t="n">
         <v>43</v>
       </c>
       <c r="B52" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="C52" s="24" t="n">
-        <v>1185433.84</v>
-      </c>
-      <c r="D52" s="22"/>
+        <v>147</v>
+      </c>
+      <c r="C52" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="D52" s="22" t="s">
+        <v>141</v>
+      </c>
       <c r="E52" s="22"/>
       <c r="F52" s="23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="11"/>
-      <c r="B53" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="11"/>
-      <c r="G53" s="11"/>
-    </row>
-    <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="25" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21" t="n">
         <v>44</v>
       </c>
-      <c r="B54" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="C54" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="D54" s="26" t="s">
+      <c r="B53" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="E54" s="26"/>
-      <c r="F54" s="27" t="s">
+      <c r="C53" s="24" t="n">
+        <v>1185433.84</v>
+      </c>
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="G53" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="G54" s="26" t="s">
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="11"/>
+      <c r="B54" s="12" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C54" s="11"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="11"/>
+      <c r="G54" s="11"/>
+    </row>
+    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="25" t="n">
         <v>45</v>
       </c>
@@ -3412,17 +3427,17 @@
         <v>153</v>
       </c>
       <c r="C55" s="26" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D55" s="26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E55" s="26"/>
       <c r="F55" s="27" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="G55" s="26" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3430,20 +3445,20 @@
         <v>46</v>
       </c>
       <c r="B56" s="26" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C56" s="26" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D56" s="26" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E56" s="26"/>
       <c r="F56" s="27" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="G56" s="26" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3451,60 +3466,81 @@
         <v>47</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C57" s="26" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D57" s="26" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="E57" s="26"/>
       <c r="F57" s="27" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="G57" s="26" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="28" t="s">
-        <v>161</v>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="25" t="n">
+        <v>48</v>
+      </c>
+      <c r="B58" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="C58" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="D58" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="E58" s="26"/>
+      <c r="F58" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="G58" s="26" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="14" t="s">
+      <c r="B60" s="28" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C60" s="5" t="n">
-        <f aca="false">COUNTIF($F$5:$F$57,B60)</f>
+      <c r="C61" s="5" t="n">
+        <f aca="false">COUNTIF($F$5:$F$58,B61)</f>
         <v>23</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="22" t="s">
-        <v>119</v>
-      </c>
-      <c r="C61" s="5" t="n">
-        <f aca="false">COUNTIF($F$5:$F$57,B61)</f>
-        <v>11</v>
-      </c>
-    </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="18" t="s">
-        <v>96</v>
+      <c r="B62" s="22" t="s">
+        <v>120</v>
       </c>
       <c r="C62" s="5" t="n">
-        <f aca="false">COUNTIF($F$5:$F$57,B62)</f>
+        <f aca="false">COUNTIF($F$5:$F$58,B62)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <f aca="false">COUNTIF($F$5:$F$58,B63)</f>
         <v>9</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="26" t="s">
-        <v>151</v>
-      </c>
-      <c r="C63" s="5" t="n">
-        <f aca="false">COUNTIF($F$5:$F$57,B63)</f>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="C64" s="5" t="n">
+        <f aca="false">COUNTIF($F$5:$F$58,B64)</f>
         <v>4</v>
       </c>
     </row>
@@ -3541,12 +3577,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3554,37 +3590,37 @@
         <v>46</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11"/>
       <c r="B5" s="12" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
@@ -3600,31 +3636,31 @@
         <v>1</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C6" s="31" t="n">
         <v>45046</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F6" s="29" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="G6" s="32" t="n">
         <v>29158.96</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="I6" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J6" s="29" t="n">
-        <v>23976</v>
+        <v>53148</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3632,31 +3668,31 @@
         <v>2</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C7" s="31" t="n">
         <v>45138</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F7" s="29" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="G7" s="32" t="n">
         <v>29158.96</v>
       </c>
       <c r="H7" s="29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="I7" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J7" s="29" t="n">
-        <v>24927</v>
+        <v>53154</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3664,31 +3700,31 @@
         <v>3</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C8" s="31" t="n">
         <v>45169</v>
       </c>
       <c r="D8" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="E8" s="29" t="s">
         <v>181</v>
       </c>
-      <c r="E8" s="29" t="s">
-        <v>176</v>
-      </c>
       <c r="F8" s="29" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="G8" s="32" t="n">
         <v>29158.96</v>
       </c>
       <c r="H8" s="29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="I8" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J8" s="29" t="n">
-        <v>25380</v>
+        <v>53156</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3696,31 +3732,31 @@
         <v>4</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C9" s="31" t="n">
         <v>45199</v>
       </c>
       <c r="D9" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="E9" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="F9" s="29" t="s">
         <v>182</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>176</v>
-      </c>
-      <c r="F9" s="29" t="s">
-        <v>177</v>
       </c>
       <c r="G9" s="32" t="n">
         <v>65819.47</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J9" s="29" t="n">
-        <v>25742</v>
+        <v>53158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3728,31 +3764,31 @@
         <v>5</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C10" s="31" t="n">
         <v>45229</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F10" s="29" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="G10" s="32" t="n">
         <v>35089.04</v>
       </c>
       <c r="H10" s="29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="I10" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J10" s="29" t="n">
-        <v>26185</v>
+        <v>53160</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3760,31 +3796,31 @@
         <v>6</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C11" s="31" t="n">
         <v>45260</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="G11" s="32" t="n">
         <v>35089.04</v>
       </c>
       <c r="H11" s="29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="I11" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J11" s="29" t="n">
-        <v>26556</v>
+        <v>53162</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3792,31 +3828,31 @@
         <v>7</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C12" s="31" t="n">
         <v>45291</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F12" s="29" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="G12" s="32" t="n">
         <v>35089.04</v>
       </c>
       <c r="H12" s="29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="I12" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J12" s="29" t="n">
-        <v>26951</v>
+        <v>53164</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3824,28 +3860,28 @@
         <v>8</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C13" s="31" t="n">
         <v>45322</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F13" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G13" s="32" t="n">
         <v>36203.78</v>
       </c>
       <c r="H13" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I13" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J13" s="29" t="n">
         <v>53166</v>
@@ -3856,28 +3892,28 @@
         <v>9</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C14" s="31" t="n">
         <v>45351</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F14" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G14" s="32" t="n">
         <v>33868.04</v>
       </c>
       <c r="H14" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I14" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J14" s="29" t="n">
         <v>53167</v>
@@ -3888,28 +3924,28 @@
         <v>10</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C15" s="31" t="n">
         <v>45382</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="E15" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F15" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G15" s="32" t="n">
         <v>37407.8</v>
       </c>
       <c r="H15" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I15" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J15" s="29" t="n">
         <v>53168</v>
@@ -3920,28 +3956,28 @@
         <v>11</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C16" s="31" t="n">
         <v>45412</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E16" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F16" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G16" s="32" t="n">
         <v>36776.27</v>
       </c>
       <c r="H16" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I16" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J16" s="29" t="n">
         <v>53169</v>
@@ -3952,28 +3988,28 @@
         <v>12</v>
       </c>
       <c r="B17" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C17" s="31" t="n">
         <v>45443</v>
       </c>
       <c r="D17" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="F17" s="29" t="s">
         <v>192</v>
-      </c>
-      <c r="E17" s="29" t="s">
-        <v>176</v>
-      </c>
-      <c r="F17" s="29" t="s">
-        <v>187</v>
       </c>
       <c r="G17" s="32" t="n">
         <v>38000.89</v>
       </c>
       <c r="H17" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I17" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J17" s="29" t="n">
         <v>53170</v>
@@ -3984,28 +4020,28 @@
         <v>13</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C18" s="31" t="n">
         <v>45473</v>
       </c>
       <c r="D18" s="29" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E18" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G18" s="32" t="n">
         <v>36106.61</v>
       </c>
       <c r="H18" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I18" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J18" s="29" t="n">
         <v>53171</v>
@@ -4016,28 +4052,28 @@
         <v>14</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C19" s="31" t="n">
         <v>45504</v>
       </c>
       <c r="D19" s="29" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="E19" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F19" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G19" s="32" t="n">
         <v>27639.77</v>
       </c>
       <c r="H19" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I19" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J19" s="29" t="n">
         <v>53172</v>
@@ -4048,28 +4084,28 @@
         <v>15</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C20" s="31" t="n">
         <v>45535</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F20" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G20" s="32" t="n">
         <v>27639.77</v>
       </c>
       <c r="H20" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I20" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J20" s="29" t="n">
         <v>53173</v>
@@ -4080,28 +4116,28 @@
         <v>16</v>
       </c>
       <c r="B21" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C21" s="31" t="n">
         <v>45565</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G21" s="32" t="n">
         <v>26748.17</v>
       </c>
       <c r="H21" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I21" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J21" s="29" t="n">
         <v>53174</v>
@@ -4112,28 +4148,28 @@
         <v>17</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C22" s="31" t="n">
         <v>45596</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="E22" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F22" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G22" s="32" t="n">
         <v>27639.77</v>
       </c>
       <c r="H22" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I22" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J22" s="29" t="n">
         <v>53177</v>
@@ -4144,28 +4180,28 @@
         <v>18</v>
       </c>
       <c r="B23" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C23" s="31" t="n">
         <v>45626</v>
       </c>
       <c r="D23" s="29" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F23" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G23" s="32" t="n">
         <v>26748.17</v>
       </c>
       <c r="H23" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I23" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J23" s="29" t="n">
         <v>53180</v>
@@ -4176,28 +4212,28 @@
         <v>19</v>
       </c>
       <c r="B24" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C24" s="31" t="n">
         <v>45657</v>
       </c>
       <c r="D24" s="29" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="E24" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="G24" s="32" t="n">
         <v>27639.77</v>
       </c>
       <c r="H24" s="29" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I24" s="29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J24" s="29" t="n">
         <v>53181</v>
@@ -4208,28 +4244,28 @@
         <v>20</v>
       </c>
       <c r="B25" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C25" s="31" t="n">
         <v>45473</v>
       </c>
       <c r="D25" s="29" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E25" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F25" s="29" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="G25" s="32" t="n">
         <v>215676.83</v>
       </c>
       <c r="H25" s="29" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="I25" s="29" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="J25" s="29" t="n">
         <v>29524</v>
@@ -4240,28 +4276,28 @@
         <v>21</v>
       </c>
       <c r="B26" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C26" s="31" t="n">
         <v>45473</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F26" s="29" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="G26" s="32" t="n">
         <v>1530000</v>
       </c>
       <c r="H26" s="29" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I26" s="29" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="J26" s="29" t="n">
         <v>36058</v>
@@ -4270,7 +4306,7 @@
     <row r="27" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11"/>
       <c r="B27" s="12" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
@@ -4286,28 +4322,28 @@
         <v>22</v>
       </c>
       <c r="B28" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C28" s="35" t="n">
         <v>44816</v>
       </c>
       <c r="D28" s="33" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="F28" s="33" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="G28" s="36" t="n">
         <v>1500000</v>
       </c>
       <c r="H28" s="33" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="I28" s="33" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="J28" s="33" t="n">
         <v>36046</v>
@@ -4318,28 +4354,28 @@
         <v>23</v>
       </c>
       <c r="B29" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C29" s="35" t="n">
         <v>44816</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="E29" s="33" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="F29" s="33" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="G29" s="36" t="n">
         <v>1500000</v>
       </c>
       <c r="H29" s="33" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="I29" s="33" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="J29" s="33" t="n">
         <v>36047</v>
@@ -4350,28 +4386,28 @@
         <v>24</v>
       </c>
       <c r="B30" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C30" s="35" t="n">
         <v>44992</v>
       </c>
       <c r="D30" s="33" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E30" s="33" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F30" s="33" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="G30" s="36" t="n">
         <v>75648.08</v>
       </c>
       <c r="H30" s="33" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="I30" s="33" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="J30" s="33" t="n">
         <v>1322</v>
@@ -4382,28 +4418,28 @@
         <v>25</v>
       </c>
       <c r="B31" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C31" s="35" t="n">
         <v>44995</v>
       </c>
       <c r="D31" s="33" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E31" s="33" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F31" s="33" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="G31" s="36" t="n">
         <v>78155.75</v>
       </c>
       <c r="H31" s="33" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="I31" s="33" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="J31" s="33" t="n">
         <v>1361</v>
@@ -4414,31 +4450,31 @@
         <v>26</v>
       </c>
       <c r="B32" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C32" s="35" t="n">
         <v>45077</v>
       </c>
       <c r="D32" s="33" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="E32" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F32" s="33" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="G32" s="36" t="n">
         <v>29158.96</v>
       </c>
       <c r="H32" s="33" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="I32" s="33" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="J32" s="33" t="n">
-        <v>24327</v>
+        <v>53150</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4446,31 +4482,31 @@
         <v>27</v>
       </c>
       <c r="B33" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C33" s="35" t="n">
         <v>45107</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E33" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F33" s="33" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="G33" s="36" t="n">
         <v>29158.96</v>
       </c>
       <c r="H33" s="33" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="I33" s="33" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="J33" s="33" t="n">
-        <v>24637</v>
+        <v>53152</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4478,28 +4514,28 @@
         <v>28</v>
       </c>
       <c r="B34" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C34" s="35" t="n">
         <v>45138</v>
       </c>
       <c r="D34" s="33" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="E34" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F34" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G34" s="36" t="n">
         <v>4082.26</v>
       </c>
       <c r="H34" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I34" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J34" s="33" t="n">
         <v>24929</v>
@@ -4510,28 +4546,28 @@
         <v>29</v>
       </c>
       <c r="B35" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C35" s="35" t="n">
         <v>45169</v>
       </c>
       <c r="D35" s="33" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F35" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G35" s="36" t="n">
         <v>4082.26</v>
       </c>
       <c r="H35" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I35" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J35" s="33" t="n">
         <v>25379</v>
@@ -4542,28 +4578,28 @@
         <v>30</v>
       </c>
       <c r="B36" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C36" s="35" t="n">
         <v>45194</v>
       </c>
       <c r="D36" s="33" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="E36" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F36" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G36" s="36" t="n">
         <v>9214.73</v>
       </c>
       <c r="H36" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I36" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J36" s="33" t="n">
         <v>25586</v>
@@ -4574,28 +4610,28 @@
         <v>31</v>
       </c>
       <c r="B37" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C37" s="35" t="n">
         <v>45224</v>
       </c>
       <c r="D37" s="33" t="s">
+        <v>242</v>
+      </c>
+      <c r="E37" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="F37" s="33" t="s">
         <v>237</v>
-      </c>
-      <c r="E37" s="33" t="s">
-        <v>176</v>
-      </c>
-      <c r="F37" s="33" t="s">
-        <v>232</v>
       </c>
       <c r="G37" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H37" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I37" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J37" s="33" t="n">
         <v>26005</v>
@@ -4606,28 +4642,28 @@
         <v>32</v>
       </c>
       <c r="B38" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C38" s="35" t="n">
         <v>45255</v>
       </c>
       <c r="D38" s="33" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="E38" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F38" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G38" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H38" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I38" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J38" s="33" t="n">
         <v>26521</v>
@@ -4638,28 +4674,28 @@
         <v>33</v>
       </c>
       <c r="B39" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C39" s="35" t="n">
         <v>45285</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="E39" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F39" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G39" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H39" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I39" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J39" s="33" t="n">
         <v>26899</v>
@@ -4670,28 +4706,28 @@
         <v>34</v>
       </c>
       <c r="B40" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C40" s="35" t="n">
         <v>45322</v>
       </c>
       <c r="D40" s="33" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="E40" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F40" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G40" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H40" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I40" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J40" s="33" t="n">
         <v>27361</v>
@@ -4702,28 +4738,28 @@
         <v>35</v>
       </c>
       <c r="B41" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C41" s="35" t="n">
         <v>45351</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F41" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G41" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H41" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I41" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J41" s="33" t="n">
         <v>27758</v>
@@ -4734,28 +4770,28 @@
         <v>36</v>
       </c>
       <c r="B42" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C42" s="35" t="n">
         <v>45382</v>
       </c>
       <c r="D42" s="33" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F42" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G42" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H42" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I42" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J42" s="33" t="n">
         <v>28283</v>
@@ -4766,28 +4802,28 @@
         <v>37</v>
       </c>
       <c r="B43" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C43" s="35" t="n">
         <v>45412</v>
       </c>
       <c r="D43" s="33" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="E43" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F43" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G43" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H43" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I43" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J43" s="33" t="n">
         <v>28840</v>
@@ -4798,28 +4834,28 @@
         <v>38</v>
       </c>
       <c r="B44" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C44" s="35" t="n">
         <v>45443</v>
       </c>
       <c r="D44" s="33" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="E44" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F44" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G44" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H44" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I44" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J44" s="33" t="n">
         <v>29301</v>
@@ -4830,28 +4866,28 @@
         <v>39</v>
       </c>
       <c r="B45" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C45" s="35" t="n">
         <v>45473</v>
       </c>
       <c r="D45" s="33" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E45" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F45" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G45" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H45" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I45" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J45" s="33" t="n">
         <v>29517</v>
@@ -4862,28 +4898,28 @@
         <v>40</v>
       </c>
       <c r="B46" s="34" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C46" s="35" t="n">
         <v>45504</v>
       </c>
       <c r="D46" s="33" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E46" s="33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F46" s="33" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G46" s="36" t="n">
         <v>4912.47</v>
       </c>
       <c r="H46" s="33" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I46" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J46" s="33" t="n">
         <v>30028</v>
@@ -4892,7 +4928,7 @@
     <row r="47" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="11"/>
       <c r="B47" s="12" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="11"/>
@@ -4908,28 +4944,28 @@
         <v>41</v>
       </c>
       <c r="B48" s="27" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C48" s="37" t="n">
         <v>44816</v>
       </c>
       <c r="D48" s="26" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="E48" s="26" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="F48" s="26" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="G48" s="38" t="n">
         <v>15030</v>
       </c>
       <c r="H48" s="26" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="I48" s="26" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="J48" s="26" t="n">
         <v>52884</v>
@@ -4940,28 +4976,28 @@
         <v>42</v>
       </c>
       <c r="B49" s="27" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C49" s="26" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D49" s="26" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="E49" s="26" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="F49" s="26" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="G49" s="38" t="n">
         <v>2981000</v>
       </c>
       <c r="H49" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="I49" s="26" t="s">
         <v>257</v>
-      </c>
-      <c r="I49" s="26" t="s">
-        <v>252</v>
       </c>
       <c r="J49" s="26" t="n">
         <v>2680</v>
@@ -4972,28 +5008,28 @@
         <v>43</v>
       </c>
       <c r="B50" s="27" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C50" s="37" t="n">
         <v>45535</v>
       </c>
       <c r="D50" s="26" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="E50" s="26" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F50" s="26" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="G50" s="38" t="n">
         <v>4912.47</v>
       </c>
       <c r="H50" s="26" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="I50" s="26" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="J50" s="26" t="n">
         <v>30592</v>
@@ -5004,28 +5040,28 @@
         <v>44</v>
       </c>
       <c r="B51" s="27" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C51" s="26" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="D51" s="26" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="E51" s="26" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="F51" s="26" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="G51" s="38" t="n">
         <v>744.96</v>
       </c>
       <c r="H51" s="26" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="I51" s="26" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="J51" s="26" t="n">
         <v>53175</v>
@@ -5033,7 +5069,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F53" s="28" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="G53" s="28" t="n">
         <f aca="false">COUNTIF(B5:B51,"DELETE")</f>
@@ -5042,7 +5078,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F54" s="28" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="G54" s="28" t="n">
         <f aca="false">COUNTIF(B5:B51,"EDIT")</f>
@@ -5051,14 +5087,14 @@
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F55" s="28" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="G55" s="39" t="n">
-        <f aca="false">SUMPRODUCT((B5:B51="EDIT")*(ISNUMBER(SEARCH("63025",F5:F51)))*G5:G51)-2*29158.96+2*4082.26</f>
+        <f aca="false">SUMIFS(G5:G51,B5:B51,"EDIT",F5:F51,"20010*63025*")+2*4082.26</f>
         <v>74668.47</v>
       </c>
       <c r="H55" s="40" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -5089,103 +5125,103 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="41" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10"/>
       <c r="B5" s="10" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
       <c r="G5" s="10"/>
       <c r="H5" s="10" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="28" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="28" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
       <c r="H10" s="10" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B11" s="42" t="n">
         <v>45456</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="D11" s="43" t="n">
         <v>109165.69</v>
@@ -5194,18 +5230,18 @@
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B12" s="42" t="n">
         <v>45456</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="D12" s="43" t="n">
         <v>106511.14</v>
@@ -5214,18 +5250,18 @@
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
       <c r="H12" s="5" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B13" s="42" t="n">
         <v>45456</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D13" s="43"/>
       <c r="E13" s="43" t="n">
@@ -5234,18 +5270,18 @@
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
       <c r="H13" s="5" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B14" s="42" t="n">
         <v>45471</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D14" s="43" t="n">
         <v>765000</v>
@@ -5254,18 +5290,18 @@
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
       <c r="H14" s="5" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B15" s="42" t="n">
         <v>45471</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D15" s="43" t="n">
         <v>765000</v>
@@ -5274,18 +5310,18 @@
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B16" s="42" t="n">
         <v>45471</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D16" s="43"/>
       <c r="E16" s="43" t="n">
@@ -5294,12 +5330,12 @@
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="5" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C17" s="12" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="D17" s="44" t="n">
         <f aca="false">SUM(D11:D16)</f>
@@ -5316,44 +5352,44 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="41" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="28" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B21" s="42" t="n">
         <v>44834</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="D21" s="43" t="n">
         <f aca="false">SUM(E21:G21)</f>
@@ -5367,18 +5403,18 @@
       </c>
       <c r="G21" s="43"/>
       <c r="H21" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="28" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B22" s="42" t="n">
         <v>44865</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="D22" s="43" t="n">
         <f aca="false">SUM(E22:G22)</f>
@@ -5392,18 +5428,18 @@
       </c>
       <c r="G22" s="43"/>
       <c r="H22" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B23" s="42" t="n">
         <v>44895</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="D23" s="43" t="n">
         <f aca="false">SUM(E23:G23)</f>
@@ -5417,18 +5453,18 @@
       </c>
       <c r="G23" s="43"/>
       <c r="H23" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="28" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="B24" s="42" t="n">
         <v>44926</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="D24" s="43" t="n">
         <f aca="false">SUM(E24:G24)</f>
@@ -5442,18 +5478,18 @@
       </c>
       <c r="G24" s="43"/>
       <c r="H24" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B25" s="42" t="n">
         <v>44957</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="D25" s="43" t="n">
         <f aca="false">SUM(E25:G25)</f>
@@ -5467,18 +5503,18 @@
       </c>
       <c r="G25" s="43"/>
       <c r="H25" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="28" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B26" s="42" t="n">
         <v>44985</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="D26" s="43" t="n">
         <f aca="false">SUM(E26:G26)</f>
@@ -5492,18 +5528,18 @@
       </c>
       <c r="G26" s="43"/>
       <c r="H26" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="28" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B27" s="42" t="n">
         <v>45016</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="D27" s="43" t="n">
         <f aca="false">SUM(E27:G27)</f>
@@ -5517,18 +5553,18 @@
       </c>
       <c r="G27" s="43"/>
       <c r="H27" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="B28" s="42" t="n">
         <v>45046</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="D28" s="43" t="n">
         <f aca="false">SUM(E28:G28)</f>
@@ -5542,18 +5578,18 @@
       </c>
       <c r="G28" s="43"/>
       <c r="H28" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="28" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B29" s="42" t="n">
         <v>45077</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D29" s="43" t="n">
         <f aca="false">SUM(E29:G29)</f>
@@ -5567,18 +5603,18 @@
       </c>
       <c r="G29" s="43"/>
       <c r="H29" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="28" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B30" s="42" t="n">
         <v>45107</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="D30" s="43" t="n">
         <f aca="false">SUM(E30:G30)</f>
@@ -5592,18 +5628,18 @@
       </c>
       <c r="G30" s="43"/>
       <c r="H30" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="28" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B31" s="42" t="n">
         <v>45138</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="D31" s="43" t="n">
         <f aca="false">SUM(E31:G31)</f>
@@ -5617,18 +5653,18 @@
       </c>
       <c r="G31" s="43"/>
       <c r="H31" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="28" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B32" s="42" t="n">
         <v>45169</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="D32" s="43" t="n">
         <f aca="false">SUM(E32:G32)</f>
@@ -5642,18 +5678,18 @@
       </c>
       <c r="G32" s="43"/>
       <c r="H32" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="28" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B33" s="42" t="n">
         <v>45199</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D33" s="43" t="n">
         <f aca="false">SUM(E33:G33)</f>
@@ -5667,18 +5703,18 @@
       </c>
       <c r="G33" s="43"/>
       <c r="H33" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B34" s="42" t="n">
         <v>45230</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="D34" s="43" t="n">
         <f aca="false">SUM(E34:G34)</f>
@@ -5692,18 +5728,18 @@
       </c>
       <c r="G34" s="43"/>
       <c r="H34" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="28" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="B35" s="42" t="n">
         <v>45260</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D35" s="43" t="n">
         <f aca="false">SUM(E35:G35)</f>
@@ -5717,18 +5753,18 @@
       </c>
       <c r="G35" s="43"/>
       <c r="H35" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="28" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B36" s="42" t="n">
         <v>45291</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="D36" s="43" t="n">
         <f aca="false">SUM(E36:G36)</f>
@@ -5742,18 +5778,18 @@
       </c>
       <c r="G36" s="43"/>
       <c r="H36" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B37" s="42" t="n">
         <v>45322</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="D37" s="43" t="n">
         <f aca="false">SUM(E37:G37)</f>
@@ -5767,18 +5803,18 @@
       </c>
       <c r="G37" s="43"/>
       <c r="H37" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="B38" s="42" t="n">
         <v>45351</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="D38" s="43" t="n">
         <f aca="false">SUM(E38:G38)</f>
@@ -5792,18 +5828,18 @@
       </c>
       <c r="G38" s="43"/>
       <c r="H38" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B39" s="42" t="n">
         <v>45382</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D39" s="43" t="n">
         <f aca="false">SUM(E39:G39)</f>
@@ -5817,18 +5853,18 @@
       </c>
       <c r="G39" s="43"/>
       <c r="H39" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="28" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B40" s="42" t="n">
         <v>45412</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="D40" s="43" t="n">
         <f aca="false">SUM(E40:G40)</f>
@@ -5842,18 +5878,18 @@
       </c>
       <c r="G40" s="43"/>
       <c r="H40" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B41" s="42" t="n">
         <v>45443</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="D41" s="43" t="n">
         <f aca="false">SUM(E41:G41)</f>
@@ -5867,18 +5903,18 @@
       </c>
       <c r="G41" s="43"/>
       <c r="H41" s="45" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B42" s="42" t="n">
         <v>45473</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D42" s="43" t="n">
         <f aca="false">SUM(E42:G42)</f>
@@ -5894,18 +5930,18 @@
         <v>581.89</v>
       </c>
       <c r="H42" s="45" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="28" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B43" s="42" t="n">
         <v>45504</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="D43" s="43" t="n">
         <f aca="false">SUM(E43:G43)</f>
@@ -5921,18 +5957,18 @@
         <v>9019.33</v>
       </c>
       <c r="H43" s="45" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="28" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B44" s="42" t="n">
         <v>45535</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="D44" s="43" t="n">
         <f aca="false">SUM(E44:G44)</f>
@@ -5948,18 +5984,18 @@
         <v>9019.33</v>
       </c>
       <c r="H44" s="45" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="28" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B45" s="42" t="n">
         <v>45565</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="D45" s="43" t="n">
         <f aca="false">SUM(E45:G45)</f>
@@ -5975,18 +6011,18 @@
         <v>8728.38</v>
       </c>
       <c r="H45" s="45" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="28" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="B46" s="42" t="n">
         <v>45596</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D46" s="43" t="n">
         <f aca="false">SUM(E46:G46)</f>
@@ -6002,18 +6038,18 @@
         <v>9019.33</v>
       </c>
       <c r="H46" s="45" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="28" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B47" s="42" t="n">
         <v>45626</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="D47" s="43" t="n">
         <f aca="false">SUM(E47:G47)</f>
@@ -6029,18 +6065,18 @@
         <v>8728.38</v>
       </c>
       <c r="H47" s="45" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="28" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B48" s="42" t="n">
         <v>45657</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="D48" s="43" t="n">
         <f aca="false">SUM(E48:G48)</f>
@@ -6056,12 +6092,12 @@
         <v>9019.33</v>
       </c>
       <c r="H48" s="45" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C49" s="12" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="D49" s="44" t="n">
         <f aca="false">SUM(D21:D48)</f>
@@ -6086,12 +6122,12 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C51" s="28" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C52" s="28" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="D52" s="43" t="n">
         <f aca="false">SUMPRODUCT((YEAR($B$21:$B$48)=2022)*D$21:D$48)</f>
@@ -6110,12 +6146,12 @@
         <v>0</v>
       </c>
       <c r="H52" s="45" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C53" s="28" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="D53" s="43" t="n">
         <f aca="false">SUMPRODUCT((YEAR($B$21:$B$48)=2023)*D$21:D$48)</f>
@@ -6134,12 +6170,12 @@
         <v>0</v>
       </c>
       <c r="H53" s="45" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C54" s="28" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="D54" s="43" t="n">
         <f aca="false">SUMPRODUCT((YEAR($B$21:$B$48)=2024)*D$21:D$48)</f>
@@ -6158,49 +6194,49 @@
         <v>54115.97</v>
       </c>
       <c r="H54" s="45" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="41" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C57" s="10" t="s">
         <v>47</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="F57" s="10" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="H57" s="10" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="28" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="B58" s="42" t="n">
         <v>44926</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="D58" s="43" t="n">
         <f aca="false">D52</f>
@@ -6218,18 +6254,18 @@
         <v>15376.5</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="28" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="B59" s="42" t="n">
         <v>45291</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="D59" s="43" t="n">
         <f aca="false">D53</f>
@@ -6247,18 +6283,18 @@
         <v>19751.95</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="28" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B60" s="42" t="n">
         <v>45657</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="D60" s="43" t="n">
         <f aca="false">D54</f>
@@ -6276,12 +6312,12 @@
         <v>24810.05</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C61" s="12" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D61" s="44" t="n">
         <f aca="false">SUM(D58:D60)</f>
@@ -6306,7 +6342,7 @@
     </row>
     <row r="63" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="46" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="B63" s="46"/>
       <c r="C63" s="46"/>
@@ -6345,34 +6381,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -6381,7 +6417,7 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="B6" s="43" t="n">
         <v>1470000</v>
@@ -6394,12 +6430,12 @@
         <v>-1470000</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B7" s="43" t="n">
         <v>0</v>
@@ -6412,12 +6448,12 @@
         <v>735000</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B8" s="43" t="n">
         <v>0</v>
@@ -6430,12 +6466,12 @@
         <v>735000</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="B9" s="43" t="n">
         <v>26536.09</v>
@@ -6448,12 +6484,12 @@
         <v>-26536.09</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="B10" s="43" t="n">
         <v>1745676.83</v>
@@ -6467,12 +6503,12 @@
         <v>0</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B11" s="43" t="n">
         <v>156337.69</v>
@@ -6486,12 +6522,12 @@
         <v>45043.9999999999</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B12" s="43" t="n">
         <v>171965.15</v>
@@ -6505,12 +6541,12 @@
         <v>29927.9099999999</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="B13" s="43" t="n">
         <v>54115.97</v>
@@ -6524,12 +6560,12 @@
         <v>0</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -6538,7 +6574,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="B15" s="43" t="n">
         <v>0</v>
@@ -6552,12 +6588,12 @@
         <v>94455.62</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="B16" s="43" t="n">
         <v>470685.22</v>
@@ -6571,12 +6607,12 @@
         <v>-101910.28</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="B17" s="43" t="n">
         <v>382418.81</v>
@@ -6590,12 +6626,12 @@
         <v>-18777.99</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="B18" s="43" t="n">
         <v>0</v>
@@ -6608,12 +6644,12 @@
         <v>40281.18</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="B19" s="43" t="n">
         <v>0</v>
@@ -6626,12 +6662,12 @@
         <v>34387.29</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="28" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="D21" s="39" t="n">
         <f aca="false">D6+D7+D8+D9+D10+D11+D12+D13</f>
@@ -6640,7 +6676,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="28" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="D22" s="39" t="n">
         <f aca="false">D15+D16+D17+D18+D19</f>
@@ -6649,24 +6685,24 @@
     </row>
     <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="34" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="D23" s="47" t="n">
         <f aca="false">ROUND(D21-D22,2)</f>
         <v>0</v>
       </c>
       <c r="E23" s="45" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="C26" s="43" t="n">
         <f aca="false">C12</f>
@@ -6675,7 +6711,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="C27" s="43" t="n">
         <v>201893.06</v>
@@ -6683,7 +6719,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="34" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="C28" s="47" t="n">
         <f aca="false">ROUND(C26-C27,2)</f>
@@ -6692,7 +6728,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="C29" s="43" t="n">
         <f aca="false">C11</f>
@@ -6701,7 +6737,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="C30" s="43" t="n">
         <v>201381.69</v>
@@ -6709,7 +6745,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="34" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="C31" s="47" t="n">
         <f aca="false">ROUND(C29-C30,2)</f>
@@ -6744,17 +6780,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="41" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6762,7 +6798,7 @@
         <v>19</v>
       </c>
       <c r="B5" s="49" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="C5" s="49"/>
       <c r="D5" s="49"/>
@@ -6774,7 +6810,7 @@
         <v>19</v>
       </c>
       <c r="B6" s="49" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="C6" s="49"/>
       <c r="D6" s="49"/>
@@ -6786,7 +6822,7 @@
         <v>19</v>
       </c>
       <c r="B7" s="49" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="C7" s="49"/>
       <c r="D7" s="49"/>
@@ -6795,158 +6831,158 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="B11" s="42" t="n">
         <v>45292</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D11" s="43" t="n">
         <v>3000000</v>
       </c>
       <c r="E11" s="43"/>
       <c r="F11" s="5" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="B12" s="42" t="n">
         <v>45292</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D12" s="43"/>
       <c r="E12" s="43" t="n">
         <v>1500000</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="B13" s="42" t="n">
         <v>45292</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D13" s="43"/>
       <c r="E13" s="43" t="n">
         <v>1500000</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="B14" s="42" t="n">
         <v>45292</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="D14" s="43" t="n">
         <v>276600.21</v>
       </c>
       <c r="E14" s="43"/>
       <c r="F14" s="5" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="B15" s="42" t="n">
         <v>45292</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="D15" s="43" t="n">
         <v>32826.52</v>
       </c>
       <c r="E15" s="43"/>
       <c r="F15" s="5" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="B16" s="42" t="n">
         <v>45292</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="D16" s="43"/>
       <c r="E16" s="43" t="n">
         <v>156352.56</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="B17" s="42" t="n">
         <v>45292</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="D17" s="43"/>
       <c r="E17" s="43" t="n">
         <v>153074.17</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="12" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D18" s="44" t="n">
         <f aca="false">SUM(D11:D17)</f>
@@ -6963,7 +6999,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6971,7 +7007,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="C21" s="49"/>
       <c r="D21" s="49"/>
@@ -6983,7 +7019,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="C22" s="49"/>
       <c r="D22" s="49"/>
@@ -6995,7 +7031,7 @@
         <v>19</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="C23" s="49"/>
       <c r="D23" s="49"/>
@@ -7007,7 +7043,7 @@
         <v>19</v>
       </c>
       <c r="B24" s="49" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="C24" s="49"/>
       <c r="D24" s="49"/>

</xml_diff>